<commit_message>
modified excel file to match desired format
</commit_message>
<xml_diff>
--- a/docs/Lab02/Lab02_BBT_TCs_Form-FINAL.xlsx
+++ b/docs/Lab02/Lab02_BBT_TCs_Form-FINAL.xlsx
@@ -121,10 +121,10 @@
     <t>Informaţiile vor fi preluate din fişiere text.</t>
   </si>
   <si>
-    <t>1. Evidenţa filmelor din colecţia personală</t>
-  </si>
-  <si>
-    <t>Un cinefil doreşte să îşi dezvolte un program pentru gestionarea filmelor din colecţia personală. Programul va permite următoarele operaţii:</t>
+    <t>1. Gestionarea unui magazin de bauturi</t>
+  </si>
+  <si>
+    <t>Un client doreste sa dezvolte o aplicatie de gestionare a unui magazin de bauturi. Aplicatia va permite următoarele operaţii:</t>
   </si>
   <si>
     <t>F01. adăugarea unui produs nou (id, nume, pret, categorie, tip);</t>
@@ -136,7 +136,7 @@
     <t xml:space="preserve">1. La proiectarea TCs se consideră o metodă care poate avea următoarea semnătură: </t>
   </si>
   <si>
-    <t>addMovie(String title, String director, int year, List&lt;String&gt; actors, String category, List&lt;String&gt; keywords): void</t>
+    <t>addProduct(int id, String name, double price, BeverageCategory categorie, BeverageType tip): void</t>
   </si>
   <si>
     <t>2. Metoda este definită la nivelul repository, service sau ui.</t>
@@ -155,17 +155,7 @@
         <color rgb="FF0070C0"/>
         <sz val="11.0"/>
       </rPr>
-      <t xml:space="preserve">Exemplu: Parametrii </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <i/>
-        <color rgb="FF0066CC"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>title</t>
+      <t>Parametrii nume</t>
     </r>
     <r>
       <rPr>
@@ -174,64 +164,7 @@
         <color rgb="FF0066CC"/>
         <sz val="11.0"/>
       </rPr>
-      <t xml:space="preserve"> şi </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <i/>
-        <color rgb="FF0066CC"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>year</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color rgb="FF0066CC"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">; Condiţii pentru aceşti parametri de intrare: </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <i/>
-        <color rgb="FF0066CC"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>title</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color rgb="FF0066CC"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> este un string cu lungimea validă de la 1 la 255 caractere; </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <i/>
-        <color rgb="FF0066CC"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>year</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color rgb="FF0066CC"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> este valid dacă ia valori între 1899 şi 2025.</t>
+      <t xml:space="preserve"> şi preț; Condiţii pentru aceşti parametri de intrare: nume este un string cu lungimea validă de la 3 la 255 caractere; preț este valid dacă ia valori întregi, mai mari decat 0(pozitive).</t>
     </r>
   </si>
   <si>
@@ -1201,16 +1134,17 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1298,6 +1232,7 @@
     <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1807,7 +1742,7 @@
       <c r="E15" s="10"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="11" t="s">
         <v>17</v>
       </c>
       <c r="C16" s="10"/>
@@ -1830,7 +1765,7 @@
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="12" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1874,14 +1809,14 @@
       <c r="O23" s="10"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
-      <c r="A24" s="14"/>
-      <c r="B24" s="15" t="s">
+      <c r="A24" s="13"/>
+      <c r="B24" s="14" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="25" ht="14.25" customHeight="1"/>
     <row r="26" ht="14.25" customHeight="1">
-      <c r="C26" s="16"/>
+      <c r="C26" s="15"/>
     </row>
     <row r="27" ht="14.25" customHeight="1"/>
     <row r="28" ht="14.25" customHeight="1"/>
@@ -2906,7 +2841,7 @@
     </row>
     <row r="2" ht="14.25" customHeight="1"/>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>25</v>
       </c>
       <c r="C3" s="2"/>
@@ -2917,13 +2852,13 @@
     </row>
     <row r="4" ht="14.25" customHeight="1"/>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="3"/>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>27</v>
       </c>
       <c r="H5" s="2"/>
@@ -2938,25 +2873,25 @@
       <c r="Q5" s="3"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="H6" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="I6" s="23" t="s">
+      <c r="I6" s="22" t="s">
         <v>34</v>
       </c>
       <c r="J6" s="2"/>
@@ -2965,54 +2900,54 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="3"/>
-      <c r="P6" s="23" t="s">
+      <c r="P6" s="22" t="s">
         <v>35</v>
       </c>
       <c r="Q6" s="3"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="B7" s="24">
+      <c r="B7" s="23">
         <v>1.0</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="24"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="28" t="s">
+      <c r="E7" s="23"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="J7" s="28" t="s">
+      <c r="J7" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="K7" s="28" t="s">
+      <c r="K7" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="L7" s="28" t="s">
+      <c r="L7" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="M7" s="28" t="s">
+      <c r="M7" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="P7" s="23" t="s">
+      <c r="P7" s="22" t="s">
         <v>42</v>
       </c>
       <c r="Q7" s="3"/>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="B8" s="24">
+      <c r="B8" s="23">
         <v>2.0</v>
       </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="26" t="s">
+      <c r="C8" s="26"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="19">
         <v>1.0</v>
       </c>
       <c r="H8" s="7" t="s">
@@ -3033,23 +2968,23 @@
       <c r="M8" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="P8" s="29" t="s">
+      <c r="P8" s="28" t="s">
         <v>48</v>
       </c>
       <c r="Q8" s="3"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
-      <c r="B9" s="24">
+      <c r="B9" s="23">
         <v>3.0</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="E9" s="24"/>
-      <c r="G9" s="20">
+      <c r="E9" s="23"/>
+      <c r="G9" s="19">
         <v>2.0</v>
       </c>
       <c r="H9" s="7">
@@ -3070,272 +3005,272 @@
       <c r="M9" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="P9" s="29" t="s">
+      <c r="P9" s="28" t="s">
         <v>51</v>
       </c>
       <c r="Q9" s="3"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
-      <c r="B10" s="24">
+      <c r="B10" s="23">
         <v>4.0</v>
       </c>
-      <c r="C10" s="31"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="26" t="s">
+      <c r="C10" s="30"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="32">
+      <c r="G10" s="31">
         <v>3.0</v>
       </c>
-      <c r="H10" s="33">
+      <c r="H10" s="32">
         <v>4.0</v>
       </c>
-      <c r="I10" s="33">
+      <c r="I10" s="32">
         <v>1.0</v>
       </c>
-      <c r="J10" s="33" t="s">
+      <c r="J10" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="K10" s="33">
+      <c r="K10" s="32">
         <v>12.0</v>
       </c>
-      <c r="L10" s="33" t="s">
+      <c r="L10" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="M10" s="33" t="s">
+      <c r="M10" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="P10" s="34" t="s">
+      <c r="P10" s="33" t="s">
         <v>54</v>
       </c>
       <c r="Q10" s="3"/>
     </row>
     <row r="11" ht="15.0" customHeight="1">
-      <c r="B11" s="24">
+      <c r="B11" s="23">
         <v>5.0</v>
       </c>
-      <c r="C11" s="27"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="26" t="s">
+      <c r="C11" s="26"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="G11" s="32">
+      <c r="G11" s="31">
         <v>4.0</v>
       </c>
-      <c r="H11" s="33">
+      <c r="H11" s="32">
         <v>5.0</v>
       </c>
-      <c r="I11" s="33">
+      <c r="I11" s="32">
         <v>1.0</v>
       </c>
-      <c r="J11" s="33" t="s">
+      <c r="J11" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="K11" s="33">
+      <c r="K11" s="32">
         <v>12.0</v>
       </c>
-      <c r="L11" s="33" t="s">
+      <c r="L11" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="M11" s="33" t="s">
+      <c r="M11" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="P11" s="34" t="s">
+      <c r="P11" s="33" t="s">
         <v>57</v>
       </c>
       <c r="Q11" s="3"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="B12" s="24">
+      <c r="B12" s="23">
         <v>6.0</v>
       </c>
-      <c r="C12" s="35" t="s">
+      <c r="C12" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="24"/>
-      <c r="G12" s="36">
+      <c r="E12" s="23"/>
+      <c r="G12" s="35">
         <v>5.0</v>
       </c>
-      <c r="H12" s="37">
+      <c r="H12" s="36">
         <v>7.0</v>
       </c>
-      <c r="I12" s="37">
+      <c r="I12" s="36">
         <v>1.0</v>
       </c>
-      <c r="J12" s="37" t="s">
+      <c r="J12" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="K12" s="37" t="s">
+      <c r="K12" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="L12" s="37" t="s">
+      <c r="L12" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="M12" s="38" t="s">
+      <c r="M12" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="P12" s="39" t="s">
+      <c r="P12" s="38" t="s">
         <v>62</v>
       </c>
       <c r="Q12" s="3"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
-      <c r="B13" s="24">
+      <c r="B13" s="23">
         <v>7.0</v>
       </c>
-      <c r="C13" s="27"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="26" t="s">
+      <c r="C13" s="26"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="G13" s="36">
+      <c r="G13" s="35">
         <v>6.0</v>
       </c>
-      <c r="H13" s="37">
+      <c r="H13" s="36">
         <v>9.0</v>
       </c>
-      <c r="I13" s="37">
+      <c r="I13" s="36">
         <v>1.0</v>
       </c>
-      <c r="J13" s="37" t="s">
+      <c r="J13" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="K13" s="37">
+      <c r="K13" s="36">
         <v>-12.0</v>
       </c>
-      <c r="L13" s="37" t="s">
+      <c r="L13" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="M13" s="37" t="s">
+      <c r="M13" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="P13" s="39" t="s">
+      <c r="P13" s="38" t="s">
         <v>64</v>
       </c>
       <c r="Q13" s="3"/>
     </row>
     <row r="14" ht="14.25" customHeight="1">
-      <c r="B14" s="24">
+      <c r="B14" s="23">
         <v>8.0</v>
       </c>
-      <c r="C14" s="40" t="s">
+      <c r="C14" s="39" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="24"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="42"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="42"/>
-      <c r="L14" s="43"/>
-      <c r="M14" s="43"/>
-      <c r="P14" s="44"/>
+      <c r="E14" s="23"/>
+      <c r="G14" s="40"/>
+      <c r="H14" s="41"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="41"/>
+      <c r="K14" s="41"/>
+      <c r="L14" s="42"/>
+      <c r="M14" s="42"/>
+      <c r="P14" s="43"/>
       <c r="Q14" s="3"/>
     </row>
     <row r="15" ht="14.25" customHeight="1">
-      <c r="B15" s="24">
+      <c r="B15" s="23">
         <v>9.0</v>
       </c>
-      <c r="C15" s="27"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="26" t="s">
+      <c r="C15" s="26"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="G15" s="41"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="42"/>
-      <c r="K15" s="42"/>
-      <c r="L15" s="42"/>
-      <c r="M15" s="42"/>
-      <c r="P15" s="45"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
+      <c r="L15" s="41"/>
+      <c r="M15" s="41"/>
+      <c r="P15" s="44"/>
       <c r="Q15" s="3"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="B16" s="24">
+      <c r="B16" s="23">
         <v>10.0</v>
       </c>
-      <c r="C16" s="46"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="42"/>
-      <c r="K16" s="42"/>
-      <c r="L16" s="42"/>
-      <c r="M16" s="42"/>
-      <c r="P16" s="45"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="41"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="41"/>
+      <c r="K16" s="41"/>
+      <c r="L16" s="41"/>
+      <c r="M16" s="41"/>
+      <c r="P16" s="44"/>
       <c r="Q16" s="3"/>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="B17" s="24">
+      <c r="B17" s="23">
         <v>11.0</v>
       </c>
-      <c r="C17" s="47"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="42"/>
-      <c r="I17" s="42"/>
-      <c r="J17" s="42"/>
-      <c r="K17" s="42"/>
-      <c r="L17" s="42"/>
-      <c r="M17" s="42"/>
-      <c r="P17" s="45"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="41"/>
+      <c r="K17" s="41"/>
+      <c r="L17" s="41"/>
+      <c r="M17" s="41"/>
+      <c r="P17" s="44"/>
       <c r="Q17" s="3"/>
     </row>
     <row r="18" ht="14.25" customHeight="1">
-      <c r="B18" s="24">
+      <c r="B18" s="23">
         <v>12.0</v>
       </c>
-      <c r="C18" s="46"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="42"/>
-      <c r="L18" s="42"/>
-      <c r="M18" s="42"/>
-      <c r="P18" s="45"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="41"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="41"/>
+      <c r="K18" s="41"/>
+      <c r="L18" s="41"/>
+      <c r="M18" s="41"/>
+      <c r="P18" s="44"/>
       <c r="Q18" s="3"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="B19" s="24">
+      <c r="B19" s="23">
         <v>13.0</v>
       </c>
-      <c r="C19" s="47"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="G19" s="20"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="G19" s="19"/>
       <c r="H19" s="6"/>
       <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
-      <c r="P19" s="45"/>
+      <c r="P19" s="44"/>
       <c r="Q19" s="3"/>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="B20" s="24">
+      <c r="B20" s="23">
         <v>14.0</v>
       </c>
-      <c r="C20" s="27"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
     </row>
     <row r="21" ht="14.25" customHeight="1"/>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="47" t="s">
         <v>68</v>
       </c>
       <c r="F22" s="48"/>
@@ -4394,7 +4329,7 @@
     </row>
     <row r="2" ht="14.25" customHeight="1"/>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="2"/>
@@ -4411,7 +4346,7 @@
       <c r="C5" s="2"/>
       <c r="D5" s="3"/>
       <c r="E5" s="50"/>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>70</v>
       </c>
       <c r="H5" s="2"/>
@@ -4427,26 +4362,26 @@
       <c r="R5" s="3"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="23" t="s">
         <v>69</v>
       </c>
       <c r="E6" s="51"/>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="H6" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="J6" s="22" t="s">
+      <c r="J6" s="21" t="s">
         <v>75</v>
       </c>
       <c r="K6" s="52" t="s">
@@ -4463,23 +4398,23 @@
       <c r="R6" s="3"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="B7" s="47">
+      <c r="B7" s="46">
         <v>1.0</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="29" t="s">
         <v>76</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
-      <c r="K7" s="28" t="s">
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="L7" s="28" t="s">
+      <c r="L7" s="27" t="s">
         <v>38</v>
       </c>
       <c r="M7" s="53" t="s">
@@ -4488,25 +4423,25 @@
       <c r="N7" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="O7" s="28" t="s">
+      <c r="O7" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="P7" s="20"/>
-      <c r="Q7" s="23" t="s">
+      <c r="P7" s="19"/>
+      <c r="Q7" s="22" t="s">
         <v>78</v>
       </c>
       <c r="R7" s="3"/>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="B8" s="31"/>
-      <c r="C8" s="31"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
       <c r="D8" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="19">
         <v>1.0</v>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="23">
         <v>1.0</v>
       </c>
       <c r="I8" s="54" t="s">
@@ -4531,18 +4466,18 @@
         <v>47</v>
       </c>
       <c r="P8" s="6"/>
-      <c r="Q8" s="29" t="s">
+      <c r="Q8" s="28" t="s">
         <v>82</v>
       </c>
       <c r="R8" s="3"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="30"/>
       <c r="D9" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="G9" s="41">
+      <c r="G9" s="40">
         <v>2.0</v>
       </c>
       <c r="H9" s="55">
@@ -4557,34 +4492,34 @@
       <c r="K9" s="57">
         <v>1.0</v>
       </c>
-      <c r="L9" s="43" t="s">
+      <c r="L9" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="M9" s="43">
+      <c r="M9" s="42">
         <v>12.0</v>
       </c>
-      <c r="N9" s="43" t="s">
+      <c r="N9" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="O9" s="43" t="s">
+      <c r="O9" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="P9" s="42"/>
-      <c r="Q9" s="39" t="s">
+      <c r="P9" s="41"/>
+      <c r="Q9" s="38" t="s">
         <v>48</v>
       </c>
       <c r="R9" s="3"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
       <c r="D10" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="19">
         <v>3.0</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="23">
         <v>3.0</v>
       </c>
       <c r="I10" s="54" t="s">
@@ -4609,21 +4544,21 @@
         <v>47</v>
       </c>
       <c r="P10" s="6"/>
-      <c r="Q10" s="29" t="s">
+      <c r="Q10" s="28" t="s">
         <v>48</v>
       </c>
       <c r="R10" s="3"/>
     </row>
     <row r="11" ht="14.25" customHeight="1">
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
       <c r="D11" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="19">
         <v>4.0</v>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="23">
         <v>4.0</v>
       </c>
       <c r="I11" s="54" t="s">
@@ -4648,21 +4583,21 @@
         <v>47</v>
       </c>
       <c r="P11" s="6"/>
-      <c r="Q11" s="29" t="s">
+      <c r="Q11" s="28" t="s">
         <v>48</v>
       </c>
       <c r="R11" s="3"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
       <c r="D12" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="19">
         <v>5.0</v>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="23">
         <v>5.0</v>
       </c>
       <c r="I12" s="54" t="s">
@@ -4685,22 +4620,22 @@
         <v>47</v>
       </c>
       <c r="P12" s="6"/>
-      <c r="Q12" s="29" t="s">
+      <c r="Q12" s="28" t="s">
         <v>48</v>
       </c>
       <c r="R12" s="3"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
-      <c r="B13" s="47">
+      <c r="B13" s="46">
         <v>2.0</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>93</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G13" s="41">
+      <c r="G13" s="40">
         <v>6.0</v>
       </c>
       <c r="H13" s="55">
@@ -4715,34 +4650,34 @@
       <c r="K13" s="57">
         <v>1.0</v>
       </c>
-      <c r="L13" s="43" t="s">
+      <c r="L13" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="M13" s="43">
+      <c r="M13" s="42">
         <v>12.0</v>
       </c>
-      <c r="N13" s="43" t="s">
+      <c r="N13" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="O13" s="43" t="s">
+      <c r="O13" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="P13" s="42"/>
-      <c r="Q13" s="39" t="s">
+      <c r="P13" s="41"/>
+      <c r="Q13" s="38" t="s">
         <v>96</v>
       </c>
       <c r="R13" s="3"/>
     </row>
     <row r="14" ht="14.25" customHeight="1">
-      <c r="B14" s="31"/>
-      <c r="C14" s="31"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
       <c r="D14" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="G14" s="20">
+      <c r="G14" s="19">
         <v>7.0</v>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="23">
         <v>7.0</v>
       </c>
       <c r="I14" s="54" t="s">
@@ -4773,15 +4708,15 @@
       <c r="R14" s="3"/>
     </row>
     <row r="15" ht="14.25" customHeight="1">
-      <c r="B15" s="31"/>
-      <c r="C15" s="31"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
       <c r="D15" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="19">
         <v>8.0</v>
       </c>
-      <c r="H15" s="24">
+      <c r="H15" s="23">
         <v>8.0</v>
       </c>
       <c r="I15" s="54" t="s">
@@ -4812,15 +4747,15 @@
       <c r="R15" s="3"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="B16" s="31"/>
-      <c r="C16" s="31"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
       <c r="D16" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="G16" s="20">
+      <c r="G16" s="19">
         <v>9.0</v>
       </c>
-      <c r="H16" s="26">
+      <c r="H16" s="25">
         <v>9.0</v>
       </c>
       <c r="I16" s="54" t="s">
@@ -4845,19 +4780,19 @@
         <v>47</v>
       </c>
       <c r="P16" s="6"/>
-      <c r="Q16" s="29" t="s">
+      <c r="Q16" s="28" t="s">
         <v>48</v>
       </c>
       <c r="R16" s="3"/>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
       <c r="D17" s="7"/>
-      <c r="G17" s="20">
+      <c r="G17" s="19">
         <v>10.0</v>
       </c>
-      <c r="H17" s="26">
+      <c r="H17" s="25">
         <v>10.0</v>
       </c>
       <c r="I17" s="54" t="s">
@@ -4882,19 +4817,19 @@
         <v>47</v>
       </c>
       <c r="P17" s="6"/>
-      <c r="Q17" s="29" t="s">
+      <c r="Q17" s="28" t="s">
         <v>102</v>
       </c>
       <c r="R17" s="3"/>
     </row>
     <row r="18" ht="14.25" customHeight="1">
-      <c r="B18" s="27"/>
-      <c r="C18" s="27"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
       <c r="D18" s="6"/>
-      <c r="G18" s="20">
+      <c r="G18" s="19">
         <v>11.0</v>
       </c>
-      <c r="H18" s="24"/>
+      <c r="H18" s="23"/>
       <c r="I18" s="62"/>
       <c r="J18" s="62"/>
       <c r="K18" s="6"/>
@@ -4907,15 +4842,15 @@
       <c r="R18" s="3"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="B19" s="47">
+      <c r="B19" s="46">
         <v>3.0</v>
       </c>
       <c r="C19" s="63"/>
       <c r="D19" s="6"/>
-      <c r="G19" s="20">
+      <c r="G19" s="19">
         <v>12.0</v>
       </c>
-      <c r="H19" s="24"/>
+      <c r="H19" s="23"/>
       <c r="I19" s="62"/>
       <c r="J19" s="62"/>
       <c r="K19" s="6"/>
@@ -4928,13 +4863,13 @@
       <c r="R19" s="3"/>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="B20" s="31"/>
-      <c r="C20" s="31"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
       <c r="D20" s="6"/>
-      <c r="G20" s="20">
+      <c r="G20" s="19">
         <v>13.0</v>
       </c>
-      <c r="H20" s="24"/>
+      <c r="H20" s="23"/>
       <c r="I20" s="62"/>
       <c r="J20" s="62"/>
       <c r="K20" s="6"/>
@@ -4947,13 +4882,13 @@
       <c r="R20" s="3"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="B21" s="31"/>
-      <c r="C21" s="31"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
       <c r="D21" s="6"/>
-      <c r="G21" s="20">
+      <c r="G21" s="19">
         <v>14.0</v>
       </c>
-      <c r="H21" s="24"/>
+      <c r="H21" s="23"/>
       <c r="I21" s="62"/>
       <c r="J21" s="62"/>
       <c r="K21" s="6"/>
@@ -4966,13 +4901,13 @@
       <c r="R21" s="3"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="B22" s="31"/>
-      <c r="C22" s="31"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
       <c r="D22" s="6"/>
-      <c r="G22" s="20">
+      <c r="G22" s="19">
         <v>15.0</v>
       </c>
-      <c r="H22" s="24"/>
+      <c r="H22" s="23"/>
       <c r="I22" s="62"/>
       <c r="J22" s="62"/>
       <c r="K22" s="6"/>
@@ -4985,13 +4920,13 @@
       <c r="R22" s="3"/>
     </row>
     <row r="23" ht="14.25" customHeight="1">
-      <c r="B23" s="31"/>
-      <c r="C23" s="31"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
       <c r="D23" s="6"/>
-      <c r="G23" s="20">
+      <c r="G23" s="19">
         <v>16.0</v>
       </c>
-      <c r="H23" s="24"/>
+      <c r="H23" s="23"/>
       <c r="I23" s="62"/>
       <c r="J23" s="62"/>
       <c r="K23" s="6"/>
@@ -5004,13 +4939,13 @@
       <c r="R23" s="3"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
       <c r="D24" s="6"/>
-      <c r="G24" s="20">
+      <c r="G24" s="19">
         <v>17.0</v>
       </c>
-      <c r="H24" s="24"/>
+      <c r="H24" s="23"/>
       <c r="I24" s="62"/>
       <c r="J24" s="62"/>
       <c r="K24" s="6"/>
@@ -5023,17 +4958,17 @@
       <c r="R24" s="3"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
-      <c r="B25" s="47">
+      <c r="B25" s="46">
         <v>4.0</v>
       </c>
       <c r="C25" s="63"/>
       <c r="D25" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="G25" s="20">
+      <c r="G25" s="19">
         <v>18.0</v>
       </c>
-      <c r="H25" s="24"/>
+      <c r="H25" s="23"/>
       <c r="I25" s="62"/>
       <c r="J25" s="62"/>
       <c r="K25" s="6"/>
@@ -5046,22 +4981,22 @@
       <c r="R25" s="3"/>
     </row>
     <row r="26" ht="14.25" customHeight="1">
-      <c r="B26" s="31"/>
-      <c r="C26" s="31"/>
+      <c r="B26" s="30"/>
+      <c r="C26" s="30"/>
       <c r="D26" s="6" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
+      <c r="B27" s="30"/>
+      <c r="C27" s="30"/>
       <c r="D27" s="6" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1">
-      <c r="B28" s="31"/>
-      <c r="C28" s="31"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="30"/>
       <c r="D28" s="6" t="s">
         <v>103</v>
       </c>
@@ -5070,8 +5005,8 @@
       <c r="N28" s="64"/>
     </row>
     <row r="29" ht="14.25" customHeight="1">
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
       <c r="D29" s="6" t="s">
         <v>103</v>
       </c>
@@ -5079,8 +5014,8 @@
       <c r="N29" s="65"/>
     </row>
     <row r="30" ht="14.25" customHeight="1">
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
       <c r="D30" s="6" t="s">
         <v>103</v>
       </c>
@@ -6150,7 +6085,7 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="20" t="s">
         <v>105</v>
       </c>
       <c r="C4" s="67" t="s">
@@ -6159,17 +6094,17 @@
       <c r="D4" s="68" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="22" t="s">
         <v>34</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="3"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="22" t="s">
         <v>35</v>
       </c>
       <c r="L4" s="3"/>
@@ -6237,7 +6172,7 @@
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="B7" s="20">
+      <c r="B7" s="19">
         <f t="shared" ref="B7:B12" si="1">B6+1</f>
         <v>2</v>
       </c>
@@ -6245,7 +6180,7 @@
       <c r="D7" s="80" t="s">
         <v>117</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="19" t="s">
         <v>112</v>
       </c>
       <c r="F7" s="76">
@@ -6271,7 +6206,7 @@
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="B8" s="20">
+      <c r="B8" s="19">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -6279,7 +6214,7 @@
       <c r="D8" s="80" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="19" t="s">
         <v>112</v>
       </c>
       <c r="F8" s="76">
@@ -6305,17 +6240,17 @@
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
-      <c r="B9" s="20">
+      <c r="B9" s="19">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C9" s="79"/>
       <c r="D9" s="81"/>
-      <c r="E9" s="20"/>
+      <c r="E9" s="19"/>
       <c r="J9" s="78"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
-      <c r="B10" s="20">
+      <c r="B10" s="19">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -6323,7 +6258,7 @@
       <c r="D10" s="81" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="27" t="s">
         <v>122</v>
       </c>
       <c r="F10" s="76">
@@ -6349,7 +6284,7 @@
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
-      <c r="B11" s="20">
+      <c r="B11" s="19">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
@@ -6357,7 +6292,7 @@
       <c r="D11" s="81" t="s">
         <v>112</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="19" t="s">
         <v>123</v>
       </c>
       <c r="F11" s="76">
@@ -6383,7 +6318,7 @@
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="B12" s="20">
+      <c r="B12" s="19">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -6391,7 +6326,7 @@
       <c r="D12" s="81" t="s">
         <v>112</v>
       </c>
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="27" t="s">
         <v>125</v>
       </c>
       <c r="F12" s="76">
@@ -6542,10 +6477,10 @@
       <c r="C19" s="93" t="s">
         <v>136</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="D19" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="E19" s="21" t="s">
+      <c r="E19" s="20" t="s">
         <v>138</v>
       </c>
       <c r="F19" s="67" t="s">
@@ -6558,16 +6493,16 @@
         <v>141</v>
       </c>
       <c r="I19" s="96"/>
-      <c r="J19" s="21" t="s">
+      <c r="J19" s="20" t="s">
         <v>136</v>
       </c>
       <c r="K19" s="97" t="s">
         <v>141</v>
       </c>
-      <c r="L19" s="21" t="s">
+      <c r="L19" s="20" t="s">
         <v>136</v>
       </c>
-      <c r="M19" s="21" t="s">
+      <c r="M19" s="20" t="s">
         <v>142</v>
       </c>
       <c r="N19" s="67" t="s">
@@ -6577,16 +6512,16 @@
     <row r="20" ht="14.25" customHeight="1">
       <c r="B20" s="98"/>
       <c r="C20" s="99"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
       <c r="F20" s="100"/>
       <c r="G20" s="101"/>
       <c r="H20" s="102"/>
       <c r="I20" s="103"/>
-      <c r="J20" s="27"/>
+      <c r="J20" s="26"/>
       <c r="K20" s="99"/>
-      <c r="L20" s="27"/>
-      <c r="M20" s="27"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
       <c r="N20" s="100"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -6629,7 +6564,7 @@
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="11" t="s">
         <v>144</v>
       </c>
       <c r="K22" s="50"/>
@@ -7615,31 +7550,31 @@
     <row r="1001" ht="14.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:G20"/>
     <mergeCell ref="H19:I20"/>
     <mergeCell ref="J19:J20"/>
+    <mergeCell ref="H21:I21"/>
     <mergeCell ref="K19:K20"/>
     <mergeCell ref="L19:L20"/>
     <mergeCell ref="M19:M20"/>
     <mergeCell ref="N19:N20"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="C6:C14"/>
     <mergeCell ref="C18:F18"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="K18:N18"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="K18:N18"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="C6:C14"/>
-    <mergeCell ref="F4:J4"/>
-    <mergeCell ref="B3:L3"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>